<commit_message>
Modificacion de documentacion y agregado de imagenes del hardware
</commit_message>
<xml_diff>
--- a/docs/Lista de Materiales.xlsx
+++ b/docs/Lista de Materiales.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365frlrutneduar-my.sharepoint.com/personal/reinoso_nery_frlr_utn_edu_ar/Documents/Proyectos/Deteccion de Caidas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365frlrutneduar-my.sharepoint.com/personal/reinoso_nery_frlr_utn_edu_ar/Documents/Proyectos/GitHub/Sistema-Monitoreo-Biomedico/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_AD4D2F04E46CFB4ACB3E20BF2510E638693EDF08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{543A9ED0-AED2-40FA-96F2-CE6CCBF53DEC}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_AD4D2F04E46CFB4ACB3E20BF2510E638693EDF08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97EC0CA2-5E72-42F8-A913-1C1AD4235204}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-4245" windowWidth="24240" windowHeight="13740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Dispositivo</t>
   </si>
@@ -183,6 +183,18 @@
   </si>
   <si>
     <t>Link de compra</t>
+  </si>
+  <si>
+    <t>ESP32 S3 Touch LCD 1.47"</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.ar/esp32-s3-touch-lcd-147-ips-con-pines-soldados-ic-de-carga/p/MLA2076646697?pdp_filters=item_id%3AMLA3178650964#polycard_client=search-desktop&amp;float_highlight=last_units&amp;be_origin=searchv2&amp;overlay_label=not_apply&amp;search_layout=grid&amp;position=31&amp;type=product&amp;tracking_id=6ebbc220-d2dd-410c-9154-f10057eb49e2&amp;wid=MLA3178650964&amp;sid=search</t>
+  </si>
+  <si>
+    <t>Pantalla Redonda TFT 1.28"</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.ar/pantalla-redonda-tft-ips-de-128-para-arduino/p/MLA57346102?pdp_filters=item_id%3AMLA2384718800#polycard_client=search-desktop&amp;be_origin=searchv2&amp;overlay_label=not_apply&amp;search_layout=grid&amp;position=1&amp;type=product&amp;tracking_id=99ad3810-ab76-4b16-8205-8c063afd1caa&amp;wid=MLA2384718800&amp;sid=search</t>
   </si>
 </sst>
 </file>
@@ -190,7 +202,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -268,19 +280,19 @@
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -562,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:E27"/>
+  <dimension ref="B2:E29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.28515625" customWidth="1"/>
@@ -802,7 +814,9 @@
       <c r="C18" s="4">
         <v>1</v>
       </c>
-      <c r="D18" s="5"/>
+      <c r="D18" s="5">
+        <v>250000</v>
+      </c>
       <c r="E18" s="4" t="s">
         <v>34</v>
       </c>
@@ -877,30 +891,58 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="10" t="s">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="9">
+        <v>41000</v>
+      </c>
+      <c r="E24" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="9">
+        <v>17500</v>
+      </c>
+      <c r="E25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11">
-        <f>SUM(D3:D23)</f>
-        <v>412000</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="10">
+        <f>SUM(D3:D25)</f>
+        <v>720500</v>
+      </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="10"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B24:C25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="B26:C27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>